<commit_message>
Remove sample answers and grading language
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R7728201bc9e9434e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="Ra2e24d3ad7b84e74"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -394,7 +394,7 @@
         <x:v>输入来源</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>虚构并脱敏的创作者后台页面、六个验收案例、发布规则、登录状态矩阵和三份storageState</x:v>
+        <x:v>虚构并脱敏的创作者后台页面、验收案例、发布规则、登录状态矩阵和storageState文件</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="66" customHeight="1">
@@ -418,7 +418,7 @@
         <x:v>目标输出文件</x:v>
       </x:c>
       <x:c r="B8" s="21" t="str">
-        <x:v>output/playwright.config.mjs；output/tests/creator_review.spec.mjs；output/reports/release_review.csv；output/receipts下的六份回执；output/screenshots下的六张页面截图</x:v>
+        <x:v>output/playwright.config.mjs；output/tests/creator_review.spec.mjs；output/reports/release_review.csv；output/receipts下的页面回执；output/screenshots下的页面截图</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="66" customHeight="1">
@@ -442,7 +442,7 @@
         <x:v>业务分支</x:v>
       </x:c>
       <x:c r="B11" s="21" t="str">
-        <x:v>核对ready_to_submit、needs_disclosure、account_limited、schedule_too_soon、needs_alt_text和reviewer_readonly六类结果及提交按钮状态</x:v>
+        <x:v>按review_scenarios.csv核对各场景的expected_state、status_text与提交按钮状态</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="56" customHeight="1">
@@ -471,33 +471,17 @@
     </x:row>
     <x:row r="15" ht="56" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>失败收口</x:v>
+        <x:v>完成条件</x:v>
       </x:c>
       <x:c r="B15" s="21" t="str">
-        <x:v>测试进程非零退出时删除本轮reports、receipts和screenshots；配置与测试源码保留，原始输入保持只读</x:v>
+        <x:v>输入场景均通过页面断言，每个case各有一份回执和一张截图，复核表业务字段与页面观察值一致，浏览器请求只指向127.0.0.1</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="56" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>完成条件</x:v>
+        <x:v>不适合作为评分点的内容</x:v>
       </x:c>
       <x:c r="B16" s="21" t="str">
-        <x:v>六个case均通过页面断言，每个case各有一份回执和一张截图，复核表业务字段与页面观察值一致，浏览器请求只指向127.0.0.1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="56" customHeight="1">
-      <x:c r="A17" s="14" t="str">
-        <x:v>可验证点</x:v>
-      </x:c>
-      <x:c r="B17" s="21" t="str">
-        <x:v>Playwright与Chromium版本；newContext的storageState；可访问定位器；业务状态和按钮；download事件；回执列和行数；截图格式；复核表路径</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="48" customHeight="1">
-      <x:c r="A18" s="14" t="str">
-        <x:v>不适合作为评分点的内容</x:v>
-      </x:c>
-      <x:c r="B18" s="21" t="str">
         <x:v>函数拆分、变量命名、测试标题、源码注释、CSV普通行序、LF或CRLF差异、截图像素级差异以及不改变规定业务结果的附加日志</x:v>
       </x:c>
     </x:row>

</xml_diff>